<commit_message>
feat(automation): integrate local machine software and implement duplicate submission protection
</commit_message>
<xml_diff>
--- a/software_service_list.xlsx
+++ b/software_service_list.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3074,6 +3074,596 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>VirtViewer</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>11.0</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Gnome / Red Hat</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>NETW2710, OSYS3030</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Open Source (Free)</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Spice protocol client for high-performance remote console access to virtual machines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Sysinternals Suite</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>OSYS1200, OSYS3030, ISEC2700</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Advanced system diagnostics utilities (Procmon, Process Explorer, Autoruns) for Windows troubleshooting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Windows Admin Center</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>OSYS1200, OSYS3030</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Free (Windows Server License Required)</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Browser-based management tool for administering Windows Server, clusters, and hyper-converged infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Windows ADK</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>NETW1500, NETW3500</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Set of tools used to customize Windows images for large-scale deployment and to test system performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Tftpd64</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Philippe Jounin</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>NETW1500, NETW3500</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Open Source (Free)</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>A lightweight IPv6-ready TFTP server and client utility used for network device firmware updates and PXE network booting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Tera Term</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>TeraTerm Project</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>NETW1027, NETW1500</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Open Source (Free)</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>A terminal emulator program supporting serial port, SSH, and telnet connections for managing switch/router consoles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>ITSM Program</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Open Source (Free)</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Local execution environment for large language models, allowing AI integration in developer tools and terminal setups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Windows Subsystem for Linux</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>2.x</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>ISEC2700, NETW2710, OSYS3030</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Compatibility layer for running Linux binary executables natively on Windows 10/11, vital for container, Docker, and DevOps labs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>WiFiman Desktop</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Ubiquiti Networks</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>NETW1027, NETW1500</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Network diagnostics tool providing Wi-Fi discovery, device scanning, and link speed analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>WinDirStat</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Bernhard Seifert</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>OSYS1200</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Open Source (Free)</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Disk usage statistics viewer and cleanup tool, helping visualize storage consumption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(automation): add MCM, WinPE, WinRE, DISM, Rufus, Ninite, Puppet, and Chef to catalog
</commit_message>
<xml_diff>
--- a/software_service_list.xlsx
+++ b/software_service_list.xlsx
@@ -452,16 +452,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
     <col width="81" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="41" customWidth="1" min="10" max="10"/>
@@ -3664,6 +3664,537 @@
         </is>
       </c>
     </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Endpoint Configuration Manager (MCM / SCCM)</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>NETW3500 (Enterprise Management and Automation)</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Subscription / Client/Server (Academic License)</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>lab, faculty, student</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Virtual Labs</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise systems management software for managing large groups of Windows-based computers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft SQL Server</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>NETW3500 (Enterprise Management and Automation), DBAS1007</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Subscription / Client/Server (Academic License / Developer Edition)</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>lab, faculty, student</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Virtual Labs</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Relational database management server, serving as the backend database host for Configuration Manager (MCM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Windows PE (Preinstallation Environment)</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>NETW1500, NETW3500</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Lightweight operating system used for preparing PCs for Windows installation and deployment (MCM dependency).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Windows Recovery Environment (WinRE)</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>OSYS1200, NETW1500</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Free (OS Native)</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Recovery environment used to troubleshoot, recover, or restore Windows installations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>DISM</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>NETW1500, NETW3500</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Free (OS Native)</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>Command-line tool used to service Windows images (.wim, .vhd) prior to deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Rufus</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Pete Batard</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>OSYS1200, NETW1500</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Open Source (Free)</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Utility that helps format and create bootable USB flash drives for OS installation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Ninite</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Secure By Design Inc.</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>OSYS1200, NETW1500</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Free / Proprietary</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, lab</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>IT Labs, Student Laptops</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>Package management utility to install and update multiple applications automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Puppet</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Puppet (Perforce)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>NETW3500 (Enterprise Management and Automation)</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Open Source / Free</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr"/>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>student, lab</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Virtual Labs, Cloud</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Configuration management utility to automate provisioning and compliance management (taught alongside Ansible).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Chef</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Progress Software</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>NETW3500 (Enterprise Management and Automation)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Open Source / Free</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr"/>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>student, lab</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Virtual Labs, Cloud</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>Infrastructure automation platform used to define infrastructure as code (taught alongside Ansible).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(automation): add Visual Studio Enterprise subscription and associated M365 and Azure environments
</commit_message>
<xml_diff>
--- a/software_service_list.xlsx
+++ b/software_service_list.xlsx
@@ -452,10 +452,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="76" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -4195,6 +4195,242 @@
         </is>
       </c>
     </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Visual Studio Enterprise Subscription</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Latest</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>ITSM Program</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Subscription (Faculty/Academic License)</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr"/>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>faculty, lab</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Online/Cloud, IT Labs</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise subscription providing access to full IDE, Azure credits, developer sandbox environments, and software licensing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Developer Sandbox</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Cloud SaaS</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>NETW3500, NETW1500</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Subscription (via VS Enterprise / Dev Program)</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, cloud</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Online/Cloud</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>A free, renewable sandboxed environment pre-configured with 25 user licenses for testing M365, Teams, Entra ID, Outlook, and Intune.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Defender for Endpoint / Cloud</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Cloud SaaS</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>ISEC2700, ISEC3700, NETW3500</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Subscription (M365 Developer / VS Enterprise)</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, cloud</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Online/Cloud</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise endpoint security platform for prevention, detection, investigation, and response.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Azure Dev Tools for Teaching (Microsoft Azure Education Hub / MS Foundry)</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Cloud SaaS</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Matt Redmond</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>IT Systems Management and Security</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>ITSM Program</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Subscription (Academic Hub)</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>student, faculty, all</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Online/Cloud</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Academic portal giving students and faculty access to software licenses (Windows Server, Windows client, SQL Server) and Azure learning resources.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>